<commit_message>
Start of RTL files
</commit_message>
<xml_diff>
--- a/docs/ISA.xlsx
+++ b/docs/ISA.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johnc\Documents\GitHub\Teensy-gpu\docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46636B90-178B-4079-A8C7-E0E354BAC5B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="25500" yWindow="0" windowWidth="25800" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,10 +24,136 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+  <si>
+    <t>Instruction Set Architecture</t>
+  </si>
+  <si>
+    <t>OP</t>
+  </si>
+  <si>
+    <t>Semantic Description</t>
+  </si>
+  <si>
+    <t>Encoding</t>
+  </si>
+  <si>
+    <t>NOP</t>
+  </si>
+  <si>
+    <t>BReq</t>
+  </si>
+  <si>
+    <t>CMP</t>
+  </si>
+  <si>
+    <t>ADDI</t>
+  </si>
+  <si>
+    <t>SUBI</t>
+  </si>
+  <si>
+    <t>MULI</t>
+  </si>
+  <si>
+    <t>DIVI?</t>
+  </si>
+  <si>
+    <t>ADDP</t>
+  </si>
+  <si>
+    <t>SUBP</t>
+  </si>
+  <si>
+    <t>MULP</t>
+  </si>
+  <si>
+    <t>DIVP</t>
+  </si>
+  <si>
+    <t>LD</t>
+  </si>
+  <si>
+    <t>ST</t>
+  </si>
+  <si>
+    <t>IMM</t>
+  </si>
+  <si>
+    <t>DONE</t>
+  </si>
+  <si>
+    <t>0000</t>
+  </si>
+  <si>
+    <t>0001</t>
+  </si>
+  <si>
+    <t>0010</t>
+  </si>
+  <si>
+    <t>0011</t>
+  </si>
+  <si>
+    <t>0100</t>
+  </si>
+  <si>
+    <t>0101</t>
+  </si>
+  <si>
+    <t>0110</t>
+  </si>
+  <si>
+    <t>0111</t>
+  </si>
+  <si>
+    <t>1000</t>
+  </si>
+  <si>
+    <t>1001</t>
+  </si>
+  <si>
+    <t>1010</t>
+  </si>
+  <si>
+    <t>1011</t>
+  </si>
+  <si>
+    <t>1100</t>
+  </si>
+  <si>
+    <t>1101</t>
+  </si>
+  <si>
+    <t>1110</t>
+  </si>
+  <si>
+    <t>1111</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -37,7 +169,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +177,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +479,222 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B2:J20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="28.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:10" ht="21" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D19" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D20" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="D3:G3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="D4:D17 D18:D19" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>